<commit_message>
111th Commit: Epic Ten Completed
</commit_message>
<xml_diff>
--- a/EPIC_0010_Report_Issues.xlsx
+++ b/EPIC_0010_Report_Issues.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Framework_For_WE1_Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3931E4D-08CE-4555-89BF-A49F9EF36036}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C318F86-BE92-4A6D-8124-DB6D70F3A93A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="31">
   <si>
     <t>Requirement Title</t>
   </si>
@@ -379,7 +379,10 @@
     <t>This test case validates the complete end-to-end booking and fulfillment flow for an Auto Ride service between the User and Driver mobile applications. It covers logging in both an approved driver and a customer with mock location set to Perambur, initiating an auto ride request to "Parsn Manere" from the User App, accepting the booking from the Driver App, extracting the ride verification OTP, updating status to "Arrived", and entering the OTP to start the trip. Finally, it verifies completing the trip, processing a cash payment settlement on both apps, and submitting mutual ratings and reviews to successfully close out the ride lifecycle.</t>
   </si>
   <si>
-    <t xml:space="preserve">1.Reload User App Completely,reload_app,user,
+    <t>TC_RG_02_Report_Issues</t>
+  </si>
+  <si>
+    <t>1.Reload User App Completely,reload_app,user,
 2.Reload Driver App Completely,reload_app,driver,
 3.Load Driver App,switch_to,driver,
 4.Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
@@ -555,11 +558,263 @@
 173.Click Add Issue Button,click,,"mobile.customer.report_issue.add_issue_btn"
 174.Wait For Issue To Load,wait,5000,
 175.Click Resolved Issue,tap_coordinate,911:716,
-176.Wait For Resolved Issue To Load,wait,5000,
-</t>
-  </si>
-  <si>
-    <t>TC_RG_02_Report_Issues</t>
+176.Wait For Resolved Issue To Load,wait,5000,</t>
+  </si>
+  <si>
+    <t>1.Reload User App Completely,reload_app,user,
+2.Reload Driver App Completely,reload_app,driver,
+3.Load Super Admin,switch_to,web,
+4.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+5.Click drivers menu,click,,"admin.drivers.menu.icon"
+6.Click Add Driver menu,click,,"admin.drivers.add_menu.link"
+7.Verify Add Driver,verify,,"admin.drivers.add_page.header"
+8.Click Service Category Dropdown,click,,"admin.drivers.service_dropdown.select"
+9.Select Auto Ride Option,click,,"admin.drivers.service_dropdown.auto_ride"
+10.Click Driver Type Dropdown,click,,"admin.drivers.driver_type.dropdown"
+11.Select pilot Option,click,,"admin.drivers.driver_type.dropdown_pilot"
+12.Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "admin.drivers.fullname.input"
+13.Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "admin.drivers.email.input"
+14.Enter Contact Number, type, {randomPhone}&gt;&gt;autoPhone, "admin.drivers.phone.input"
+15.Click Whatspp, click, , "admin.drivers.whatsapp.checkbox"
+16.Enter Whatspp Number, type, {autoPhone}, "admin.drivers.whatsapp_phone.input"
+17.Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "admin.drivers.profile_image.file"
+18.Select Source,click,,"admin.drivers.source_dropdown.select"
+19.Select Instagram,click,,"admin.drivers.instagram_option.span"
+20.Select Male Gender, click, , "admin.drivers.male_gender.div"
+21.Click Vehicle Type Dropdown,click,,"admin.drivers.vehicle_dropdown.select"
+22. Select  Auto Option,click,,"admin.drivers.vehicle_option.pinkauto"
+23. Enter Model Year, type, 2013, "admin.drivers.modelyear.input"
+24. Enter Plate No, type, KL-01-AB-1234, "admin.drivers.plateno.input"
+25. Enter Model Name, type, petrol, "admin.drivers.modelname.input"
+26. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "admin.drivers.vehicle_image.file"
+27. Enter Bank Name, type, HDFC Bank, "admin.drivers.bankname.input"
+28. Enter Bank Location, type, PARK STREET, "admin.drivers.banklocation.input"
+29. Enter Account Number, type, 50100123456789, "admin.drivers.accountno.input"
+30. Enter Account Holder Name, type,{autoName}, "admin.drivers.accountholder.input"
+31. Enter Payment Email Address, type, {autoEmail}, "admin.drivers.paymentemail.input"
+32. Enter IFSC Code, type, HDFC0001234, "admin.drivers.ifsc.input"
+33. Click Submit, click, , "web.global.action.submit"
+34. Verify Driver Added, verify,, "web.global.toast.success"
+35. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+36. Click drivers menu,click,,"admin.drivers.menu.icon"
+37. Click Pending Documents,click,,"admin.drivers.pending_docs.link"
+38. Filter by Name,type,{autoName},"admin.drivers.name_filter.input"
+39. Scroll Grid, tab, 7, "admin.drivers.name_filter.input"
+40. Click Doc Icon,click,,"admin.drivers.docs.icon"
+41. Driver Required Documents,verify,,"admin.drivers.required_docs.header"
+42. FilterDocumet List,type,Driving Licence,"admin.drivers.docs_filter.input"
+43. Add Driving License,click,,"admin.drivers.docs.edit_icon"
+44. Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "admin.drivers.profile_image.file"
+45. Enter Expiry Date,set_date,2026-12-12,"admin.drivers.doc_expiry.input"
+46. Click Submit, click, , "web.global.action.submit"
+47. Verify Updated Succesfully, verify, , "web.global.toast.updated"
+48. Click Approve Driver,click,,"admin.drivers.docs.approval"
+49. Verify Updated Succesfully, verify, , "web.global.toast.updated"
+50. Click Dashboard,click,,"web.global.menu.dashboard"
+51. Click drivers menu,click,,"admin.drivers.menu.icon"
+52. Click Approved Drivers,click,,"admin.drivers.approved_docs.link"
+53. Approved Drivers List,verify,,"admin.drivers.approved_page.header"
+54. Filter Approved Driver,type,{autoName},"admin.drivers.name_filter.input"
+55.Wait For Load,wait,2000,
+56.Scroll Grid,tab,10,"admin.drivers.name_filter.input"
+57.Click Wallet,click,,"admin.drivers.wallet.btn"
+58.Click Manage Transaction,click,,"admin.drivers.wallet.manage_transaction.btn"
+59.Enter Wallet Amout,type,500,"admin.drivers.wallet.wallet_amount_input"
+60.Click Dropdown,click,,"admin.drivers.wallet.option_dropdown"
+61.Select Add Money Optin,click,,"admin.drivers.wallet.option_add_money"
+62.Click Submit Button,click,,"admin.drivers.wallet.submit.btn"
+63.Wait For Recharge,wait,2000,
+64. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+65.Click Customer Icon,click,,"admin.menu.customer_icon"
+66.Click Add Customers,click,,"admin.menu.add_customers"
+67.Wait For Customer Heading,wait_until_visible,,"admin.customer.add_heading"
+68.Enter Customer Name,type,customer{randomAlpha} &gt;&gt; customerName,"admin.customer.input_name"
+69.Enter Email,type,customer_{timestamp}@gmail.com&gt;&gt;customerEmail,"admin.customer.input_email"
+70.Enter Contact Number,type,{randomPhone}&gt;&gt;customerPhone,"admin.customer.input_phone"
+71.Enter Emergency Number,type,{randomPhone},"admin.customer.input_Emergency_phone"
+72.Open Gender,click,,"admin.customer.dropdown_gender"
+73.Select Male,click,,"admin.customer.select_gender_male"
+74.Upload Profile Image,uploadfile,"src/main/resources/test-data/customer.jpg","admin.customer.upload_profile_img"
+75.Click Submit,click,,"web.global.action.submit"
+76.Wait For Added Successfully,wait_until_visible,,"web.global.toast.info"
+77.Click Dashboard,click,,"web.global.menu.dashboard"
+78.Click Customer Icon,click,,"admin.menu.customer_icon"
+79.Click Verified Customers,click,,"admin.menu.verified_customers"
+80.Wait For Customer List Heading,wait_until_visible,,"admin.customer.verified_list_heading"
+81.Filter Customer Name List,type,{customerName},"admin.customer.filter_name"
+82.Wait For Load,wait,2000,
+83.Load Driver App,switch_to,driver,
+84.Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+85.Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+86.Click Agree,tap,,"mobile.driver.agree.btn"
+87. Click Get Started,tap,,"mobile.driver.get_started.btn"
+88.Click Next,tap,,"mobile.driver.next.btn"
+89.Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+90.Click Close,tap,,"mobile.driver.cancel.btn"
+91. Enter Mobile Number,type,{autoPhone},"mobile.driver.edit_text.input"
+92.Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+93.Click Continue,tap,,"mobile.driver.continue.btn"
+94.Enter OTP,type,123456,"mobile.driver.edit_text.input"
+95.Enter Account Holder,type,{autoName},"mobile.driver.bank_details.account_holder_name"
+96.Enter Account Number,type,50100123456789,"mobile.driver.bank_details.account_number"
+97.Enter Confirm Account Number,type,50100123456789,"mobile.driver.bank_details.confirm_account_number"
+98.Enter IFSC Code,type,HDFC0001234,"mobile.driver.bank_details.confirm_ifsc_code"
+99.Wait For Keyboard Minimises,hide_keyboard,, 
+100.Enter Upi Id,type,sujanpariyar07@fam,"mobile.driver.bank_details.upi_id"
+101.Wait For Keyboard Minimises,hide_keyboard,,
+102.Click Submit,click,,"mobile.driver.bank_details.submit_btn"
+103.Force Driver Location To Perambur,set_location,13.121030;80.232578,
+104.Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+105.Wait for Toast to Hide,wait,3000,,
+106.Click Select All Agree,tap,,"mobile.driver.independent_contractor.checkbox_Select_All"
+107.Wait for Agree,wait_until_visible,,"mobile.driver.agree_continue.btn"
+108.Click Agree,tap,,"mobile.driver.agree_continue.btn"
+109.Wait For OTP,wait_until_visible,,"mobile.driver.edit_text.input"
+110. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+111. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+112.Wait For Hamburger Menu,wait,3000
+113.Click Online Toggle,tap_coordinate ,975:1935,COORDINATE_MODE
+114.wait for page load,wait,3000,
+115.Load User App,switch_to,user,
+116.Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
+117.Click Get Started,tap,,"mobile.customer.get_started.btn"
+118.Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
+119.Force User Location To Perambur,set_location,13.121030;80.232578,
+120.Click Next,tap,,"mobile.customer.next.btn"
+121.Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+122.Click Close,tap,,"mobile.customer.cancel.btn"
+123.Enter Mobile Number,type,{customerPhone},"mobile.customer.edit_text.input"
+124.Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
+125.Click Continue,tap,,"mobile.customer.continue.btn"
+126.Enter OTP,type,123456,"mobile.customer.otp_input"
+127.Wait for Finish,wait_until_visible,,"mobile.customer.finish.btn"
+128.Click Finish,tap,,"mobile.customer.finish.btn"
+129.Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+130.Wait For Auto Ride,wait_until_visible,,"mobile.customer.auto_ride.btn"
+131.Click Auto Ride,tap,,"mobile.customer.auto_ride.btn"
+132.Enter Destination,type,Parsn Manare,"mobile.customer.destination.input"
+133.Wait for Location,wait_until_visible,,"mobile.customer.set_location_map.btn"
+134.Select Destination,tap,,"mobile.customer.destination_suggestion_first"
+135.Wait For Entrance,wait_until_visible,,"mobile.customer.destination_entrance_location"
+136.Click Entrance,tap,,"mobile.customer.destination_entrance_location"
+137.Click Confirm,tap,,"mobile.customer.confirm.btn"
+138.Wait For Ride,wait,5000,
+139.Wait for Ride,wait_until_visible,,"mobile.customer.ride_now.btn"
+140.Ride Now,tap,,"mobile.customer.ride_now.btn"
+141.Load Driver App,switch_to,driver,
+142.Wait for Accept,wait_until_visible,,"mobie.driver.auto_ride_accept.button"
+143.Click  Accept Ride,tap,,"mobie.driver.auto_ride_accept.button"
+144.Load User App,switch_to,user,
+145.Wait for OTP Layout to Load,wait_until_visible,,"mobile.customer.otp_display_element"
+146.Extract OTP from Screen,store_text,ride_otp,"mobile.customer.otp_display_element"
+147.Load Driver App,switch_to,driver,
+148.Wait for On My Way,wait_until_visible,,"mobile.driver.on_my_way.btn"
+149.Wait for Arrived,wait_until_visible,,"mobile.driver.arrived.btn"
+150.Wait for Arrived,wait_until_visible,,"mobile.driver.arrived.btn"
+151.Ride Arrived,tap,,"mobile.driver.arrived.btn"
+152.Wait for Yes,wait_until_visible,,"mobile.driver.yes.btn"
+153.Yes Arrived,tap,,"mobile.driver.yes.btn"
+154.Wait for Start Ride,wait_until_visible,,"mobile.driver.start_ride.btn"
+155.Start Ride,tap,,"mobile.driver.start_ride.btn"
+156.wait for Otp,wait_until_visible,,"mobile.driver.otp_view.input"
+157.Enter  Extracted OTP,type,{ride_otp},"mobile.driver.otp_view.input"
+158.Wait for Start Button,wait_until_visible,,"mobile.driver.start.btn"
+159.Start Ride Button,tap,,"mobile.driver.start.btn"
+160.Wait for Complete Ride,wait_until_visible,,"mobile.driver.complete_ride.btn"
+161.Complete Ride,tap,,"mobile.driver.complete_ride.btn"
+162.Wait for Collect Payment,wait_until_visible,,"mobile.driver.collect_payment.btn"
+163.Collect Payment,tap,,"mobile.driver.collect_payment.btn"
+164.Load User App,switch_to,user,
+165.Wait for Proceed Payment,wait_until_visible,,"mobile.customer.proceed_to_pay.btn"
+166.Proceed Payment,tap,,"mobile.customer.proceed_to_pay.btn"
+167.Wait for Proceed Pay Confirm,wait_until_visible,,"mobile.customer.proceed_to_pay.btn"
+168.Pay Cash,tap,,"mobile.customer.proceed_to_pay.btn"
+169.Wait for Review,wait_until_visible,,"mobile.customer.give_review.btn"
+170.Give Review,tap,,"mobile.customer.give_review.btn"
+171.Give Rating,tap_coordinate,348:1619,
+172.Submit Rating,tap,,"mobile.customer.submit_rating.btn"
+173.Wait for Done,wait_until_visible,,"mobile.customer.done.btn"
+174.Trip Finished,tap,,"mobile.customer.done.btn"
+175. Load Driver App,switch_to,driver,
+176.Wait  For Proceed,wait_until_visible,,"mobile.driver.payment.proceed_btn"
+177.Click For Proceed,tap,,"mobile.driver.payment.proceed_btn"
+178.Wait for Yes,wait_until_visible,,"mobile.driver.yes.btn"
+179.Confirm Payment,tap,,"mobile.driver.yes.btn"
+180.Wait For Give Review Button,wait_until_visible,,"mobile.driver.give_review.btn"
+181.Click Give Review Button,tap,,"mobile.driver.give_review.btn"
+182.Wait For Rating,wait,2000,
+183.Give Rating,tap_coordinate,348:1545,
+184.Submit Rating,tap,,"mobile.driver.submit_rating.btn"
+185.Wait for Complete Button,wait_until_visible,,"mobile.driver.complete.btn"
+186.Click Complete Button,tap,,"mobile.driver.complete.btn"
+187.Wait For  ride complete submit button,wait_until_visible,,"mobile.driver.ride_complete_submit.btn"
+188.Click Ride Complete Submit Button,tap,,"mobile.driver.ride_complete_submit.btn"
+189.Load User App,switch_to,user,
+190.Wait for Back,wait_until_visible,,"mobile.customer.back.btn"
+191.Click Back Button,tap,,"mobile.customer.back.btn"
+192. Wait For Landing Page,wait_until_visible,,"mobile.customer.home_page.profile_icon"
+193.Click Profile Menu,tap,,"mobile.customer.home_page.profile_icon"
+194.Wait For Profile,wait_until_visible,,"mobile.customer.account.heading"
+195.Click My Orders,tap,,"mobile.customer.profile.my_orders_btn"
+196.Wait For My Orders Heading,wait_until_visible,,"mobile.customer.profile.my_orders_heading"
+197.Wait For Orders To Load,wait,3000,
+198.Click Completed Ride,tap_coordinate,532:961,
+199.Wait For Three Dot Menu,wait_until_visible,,"mobile.customer.my_orders.three_dot_menu"
+200.Click Three Dot Menu,tap,,"mobile.customer.my_orders.three_dot_menu"
+201.Click Report Issue Popup,tap,,"mobile.customer.my_orders.report_issue"
+202.Type Issue Description,type,Bad Behaviour Of Driver,"mobile.customer.my_orders.report_issue.description_fld"
+203.Click Add Image,tap,,"mobile.customer.my_orders.report_issue.add_image"
+204.Click Camera  Icon,tap,,"mobile.customer.my_orders.report_issue.add_image_camera"
+205.Click Allow Notification,tap_if_present,,"mobile.customer.my_orders.report_issue.camera_allow_notification"
+206.Wait For Camera Shutter,wait_until_visible,,"mobile.customer.my_orders.report_issue.add_image_camera_shutter"
+207.Clilck Camera Shutter,tap,,"mobile.customer.my_orders.report_issue.add_image_camera_shutter"
+208.Wait For Done,wait_until_visible,,"mobile.customer.my_orders.report_issue.add_image_done"
+209.Click Done,tap,,"mobile.customer.my_orders.report_issue.add_image_done"
+210.Wait For Crop,wait_until_visible,,"mobile.customer.my_orders.report_issue.crop_done"
+211.Click Crop,tap,,"mobile.customer.my_orders.report_issue.crop_done"
+212.Wait For Submit Issue Button,wait_until_visible,,"mobile.customer.my_orders.report_issue.submit_issue_btn"
+213.Click Submit Issue Button,tap,,"mobile.customer.my_orders.report_issue.submit_issue_btn"
+214.Wait For Report Issue Chat Button,wait_until_visible,,"mobile.customer.my_orders.report_issue.chat_btn"
+215.Extract Ticket ID From Ui,store_text,ticket_id,"mobile.customer.my_orders.report_issue.ticket_id_field"
+216.Click Chat Button,tap,,"mobile.customer.my_orders.report_issue.chat_btn"
+217.Wait For Chat Box,wait_until_visible,,"mobile.customer.my_orders.report_issue.chat_box"
+218.Type Chat,type,Hi today had an bad experince from your driver with above ride id please look into it take necessary action thank you,"mobile.customer.my_orders.report_issue.chat_box"
+219.Enter Chat,tap,,"mobile.customer.my_orders.report_issue.chat_box_enter_btn"
+220.Switch To Web Session,switch_to,web,
+221.Click Dashboard,click,,"web.global.menu.dashboard"
+222.Wait To Load,wait,2000,
+223.Click Bell Icon,click,, "web.global.btn_notification_bell"
+224. Click Report Issue Flag,click,, "web.global.btn_report_issue_flag"
+225. Click  Customer Notificaton,click,, "web.global.item_report_alert_by_customer"
+226. Close  Global Alert,click,, "web.global.btn_close_report_alerts"
+227. Scroll Grid,tab,8, "admin.report_issue.customer_report_issues.ticket_id_filter_input"
+228.Wait For Grid Load,wait,2000,
+229.View Eye Icon,click,,"admin.report_issue.customer_report_issues.eye_icon"
+230.Close Eye Icon,click,,"admin.report_issue.customer_report_issues.close_eye_icon"
+231.Click Chat Icon,click,,"admin.report_issue.customer_report_issues.chat_icon"
+232.Reply Customer Issue,type,Thank you for raising the issue strict action will be taken against the driver we apolgize for inconvince,"admin.report_issue.customer_report_issues.chat_box"
+233.Click Enter Chat,click,,"admin.report_issue.customer_report_issues.chat_box_enter_btn"
+234.Close Chat Box,click,,"admin.report_issue.customer_report_issues.close_chat_icon"
+235.Click Resolved Issue,click,,"admin.report_issue.customer_report_issues.resolve_thumbs_icon"      
+236.Confirm Resolved Issue,click,,"admin.report_issue.customer_report_issues.resolve_confirm_yes"
+237.Load User App,switch_to,user,
+238.Wait For Chat Box,wait_until_visible,,"mobile.customer.my_orders.report_issue.chat_box"
+239.Click Back Button,tap,,"mobile.customer.my_orders.report_issue.back_btn"
+240.Wait For Chat Button,wait_until_visible,,"mobile.customer.my_orders.report_issue.chat_btn"
+241.Click Back Button,tap,,"mobile.customer.my_orders.report_issue.back_btn"
+242.Wait For Three Dot Menu,wait_until_visible,,"mobile.customer.my_orders.three_dot_menu"
+243.Click Back Button,tap,,"mobile.customer.my_orders.report_issue.back_btn"
+244.Wait for My Orders Heading,wait_until_visible,,"mobile.customer.profile.my_orders_heading" 
+245.Click Back Button,tap,,"mobile.customer.my_orders.report_issue.back_btn"
+246.Wait For  Profile Load,wait,2000,
+247.Swipe Up Page,swipe,up,
+248.Wait For Profile Load,wait,2000, 
+249.Click Report Issue,click,,"mobile.customer.profile.report_issue"
+250.Wait for Add Issue,wait_until_visible,,"mobile.customer.report_issue.add_issue_btn" 
+251.Click Add Issue Button,click,,"mobile.customer.report_issue.add_issue_btn"
+252.Wait For Issue To Load,wait,5000,
+253.Click Resolved Issue,tap_coordinate,911:716,
+254.Wait For Resolved Issue To Load,wait,5000,</t>
   </si>
 </sst>
 </file>
@@ -1012,10 +1267,10 @@
     <col min="4" max="4" width="28.77734375" customWidth="1"/>
     <col min="5" max="5" width="29.109375" customWidth="1"/>
     <col min="6" max="6" width="45.77734375" customWidth="1"/>
-    <col min="7" max="7" width="71.44140625" customWidth="1"/>
+    <col min="7" max="7" width="69.33203125" customWidth="1"/>
     <col min="8" max="8" width="40.44140625" customWidth="1"/>
-    <col min="9" max="9" width="61.88671875" customWidth="1"/>
-    <col min="10" max="10" width="32.88671875" customWidth="1"/>
+    <col min="9" max="9" width="32.77734375" customWidth="1"/>
+    <col min="10" max="10" width="62" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
@@ -1061,7 +1316,7 @@
         <v>20</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>27</v>
@@ -1070,7 +1325,7 @@
         <v>26</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
@@ -1078,7 +1333,9 @@
       <c r="I2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="J2" s="2"/>
+      <c r="J2" s="2" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>

</xml_diff>